<commit_message>
Finance : modèles financiers remplis (données disponibles + hypothèses temporaires) et fiche des données manquantes (27/10/2026)
Prévisions restructurées sur l'offre Fou d'un soir (Premier soir, Le Voyage,
La Grande Nuit, privatisation) avec TVA, capacité et remplissage ; financement
et trésorerie en hypothèses (H), aucun fait comptable. La fiche liste
19 données manquantes, l'hypothèse retenue et le pôle qui peut la fournir.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/2 FINANCE/FINANCEMENT/2026 1027 Modèle - Financement et table de capitalisation.xlsx
+++ b/2 FINANCE/FINANCEMENT/2026 1027 Modèle - Financement et table de capitalisation.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vians\Documents\Claude\Projects\HEC-GEMM-Groupe-7\2 FINANCE\FINANCEMENT\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{52086631-14D7-4949-B3A8-366D19CCD864}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73FB2527-5156-453A-AB5F-C9FAB5C384E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{C6848D91-B8BF-4AD6-8B0B-F91FE7845E07}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="144">
   <si>
     <t>Financement — levées de fonds, prêts, subventions, table de capitalisation</t>
   </si>
@@ -382,6 +382,99 @@
   </si>
   <si>
     <t>Non modélisé : préférence de liquidation, anti-dilution, création d'un nouveau plan de BSPCE. Les lire dans les pièces avant de calculer ce que chaque associé reçoit.</t>
+  </si>
+  <si>
+    <t>État du fichier</t>
+  </si>
+  <si>
+    <t>Mis à jour le 27/10/2026 : aucune donnée de financement n'existe dans le dépôt (ni apport, ni demande, ni pièce). Toutes les valeurs saisies sont des hypothèses temporaires (H), au statut « Envisagé » : le total reçu reste à 0 €. Voir 2 FINANCE/2026 1027 Données financières manquantes et hypothèses temporaires.md.</t>
+  </si>
+  <si>
+    <t>[associés fondateurs, 7 membres de l'équipe]</t>
+  </si>
+  <si>
+    <t>Capital social de 7 000 € : 1 000 € par associé</t>
+  </si>
+  <si>
+    <t>Hypothèse temporaire ; nombre d'associés repris de README.md (sept fonctions, un responsable par fonction) ; montant à fixer par les associés</t>
+  </si>
+  <si>
+    <t>[réseau d'accompagnement à la création]</t>
+  </si>
+  <si>
+    <t>Prêt personnel aux fondateurs, taux zéro, 5 ans (H)</t>
+  </si>
+  <si>
+    <t>Hypothèse temporaire ; couvre le besoin de l'année 1 du plan financier (2 FINANCE/PREVISIONS)</t>
+  </si>
+  <si>
+    <t>[concours ou incubateur]</t>
+  </si>
+  <si>
+    <t>À identifier</t>
+  </si>
+  <si>
+    <t>Hypothèse temporaire ; aucun dispositif identifié dans le dépôt</t>
+  </si>
+  <si>
+    <t>[business angels, dont l'associé gastronomique envisagé]</t>
+  </si>
+  <si>
+    <t>Augmentation de capital, voir onglet « Après levée »</t>
+  </si>
+  <si>
+    <t>Hypothèse temporaire ; l'associé gastronomique au capital est évoqué dans 1 DIRECTION/STRATEGIE/2026 1027 Fiche de synthèse du projet (proposition, non décidée)</t>
+  </si>
+  <si>
+    <t>Aucune : prêt non signé, simulation</t>
+  </si>
+  <si>
+    <t>Hypothèse temporaire (ligne 2 du suivi des financements)</t>
+  </si>
+  <si>
+    <t>Aucune : statuts non rédigés, société non créée (hypothèse temporaire)</t>
+  </si>
+  <si>
+    <t>Associé fondateur (Direction)</t>
+  </si>
+  <si>
+    <t>Actions ordinaires</t>
+  </si>
+  <si>
+    <t>Aucun</t>
+  </si>
+  <si>
+    <t>Aucune</t>
+  </si>
+  <si>
+    <t>Associé fondateur (Finance)</t>
+  </si>
+  <si>
+    <t>Associé fondateur (Marketing)</t>
+  </si>
+  <si>
+    <t>Associé fondateur (Ventes)</t>
+  </si>
+  <si>
+    <t>Associé fondateur (Produit)</t>
+  </si>
+  <si>
+    <t>Associé fondateur (Opérations)</t>
+  </si>
+  <si>
+    <t>Associé fondateur (Juridique)</t>
+  </si>
+  <si>
+    <t>Business angels, dont un associé gastronomique (H)</t>
+  </si>
+  <si>
+    <t>Hypothèse temporaire, aucune évaluation ; à fonder sur les premiers résultats des pilotes</t>
+  </si>
+  <si>
+    <t>Hypothèse temporaire ; ordre de grandeur du besoin cumulé du plan à 3 ans (2 FINANCE/PREVISIONS)</t>
+  </si>
+  <si>
+    <t>1 DIRECTION/STRATEGIE/2026 1027 Fiche de synthèse du projet, § Associé gastronomique (proposition)</t>
   </si>
 </sst>
 </file>
@@ -614,9 +707,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="167" fontId="8" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="167" fontId="9" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -624,6 +714,9 @@
     <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="6" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -958,7 +1051,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B54AE698-D5A6-4B60-8701-006A5958E622}">
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.6328125" style="1" customWidth="1"/>
@@ -1078,6 +1171,14 @@
       </c>
       <c r="B16" s="7" t="s">
         <v>27</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A17" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="B17" s="7" t="s">
+        <v>114</v>
       </c>
     </row>
   </sheetData>
@@ -1195,76 +1296,132 @@
         <v>53</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:14" ht="62.5" x14ac:dyDescent="0.25">
       <c r="A6" s="7">
         <v>1</v>
       </c>
-      <c r="B6" s="18"/>
-      <c r="C6" s="18"/>
+      <c r="B6" s="18" t="s">
+        <v>62</v>
+      </c>
+      <c r="C6" s="18" t="s">
+        <v>115</v>
+      </c>
       <c r="D6" s="19"/>
-      <c r="E6" s="20"/>
-      <c r="F6" s="18"/>
+      <c r="E6" s="20">
+        <v>7000</v>
+      </c>
+      <c r="F6" s="18" t="s">
+        <v>49</v>
+      </c>
       <c r="G6" s="20"/>
       <c r="H6" s="20"/>
       <c r="I6" s="19"/>
       <c r="J6" s="18"/>
-      <c r="K6" s="18"/>
-      <c r="L6" s="18"/>
-      <c r="M6" s="18"/>
+      <c r="K6" s="18" t="s">
+        <v>116</v>
+      </c>
+      <c r="L6" s="18" t="s">
+        <v>51</v>
+      </c>
+      <c r="M6" s="18" t="s">
+        <v>117</v>
+      </c>
       <c r="N6" s="18"/>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:14" ht="37.5" x14ac:dyDescent="0.25">
       <c r="A7" s="7">
         <v>2</v>
       </c>
-      <c r="B7" s="18"/>
-      <c r="C7" s="18"/>
+      <c r="B7" s="18" t="s">
+        <v>45</v>
+      </c>
+      <c r="C7" s="18" t="s">
+        <v>118</v>
+      </c>
       <c r="D7" s="19"/>
-      <c r="E7" s="20"/>
-      <c r="F7" s="18"/>
+      <c r="E7" s="20">
+        <v>20000</v>
+      </c>
+      <c r="F7" s="18" t="s">
+        <v>49</v>
+      </c>
       <c r="G7" s="20"/>
       <c r="H7" s="20"/>
       <c r="I7" s="19"/>
       <c r="J7" s="18"/>
-      <c r="K7" s="18"/>
-      <c r="L7" s="18"/>
-      <c r="M7" s="18"/>
+      <c r="K7" s="18" t="s">
+        <v>119</v>
+      </c>
+      <c r="L7" s="18" t="s">
+        <v>51</v>
+      </c>
+      <c r="M7" s="18" t="s">
+        <v>120</v>
+      </c>
       <c r="N7" s="18"/>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:14" ht="25" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
         <v>3</v>
       </c>
-      <c r="B8" s="18"/>
-      <c r="C8" s="18"/>
+      <c r="B8" s="18" t="s">
+        <v>65</v>
+      </c>
+      <c r="C8" s="18" t="s">
+        <v>121</v>
+      </c>
       <c r="D8" s="19"/>
-      <c r="E8" s="20"/>
-      <c r="F8" s="18"/>
+      <c r="E8" s="20">
+        <v>5000</v>
+      </c>
+      <c r="F8" s="18" t="s">
+        <v>49</v>
+      </c>
       <c r="G8" s="20"/>
       <c r="H8" s="20"/>
       <c r="I8" s="19"/>
       <c r="J8" s="18"/>
-      <c r="K8" s="18"/>
-      <c r="L8" s="18"/>
-      <c r="M8" s="18"/>
+      <c r="K8" s="18" t="s">
+        <v>122</v>
+      </c>
+      <c r="L8" s="18" t="s">
+        <v>51</v>
+      </c>
+      <c r="M8" s="18" t="s">
+        <v>123</v>
+      </c>
       <c r="N8" s="18"/>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:14" ht="75" x14ac:dyDescent="0.25">
       <c r="A9" s="7">
         <v>4</v>
       </c>
-      <c r="B9" s="18"/>
-      <c r="C9" s="18"/>
+      <c r="B9" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="C9" s="18" t="s">
+        <v>124</v>
+      </c>
       <c r="D9" s="19"/>
-      <c r="E9" s="20"/>
-      <c r="F9" s="18"/>
+      <c r="E9" s="20">
+        <v>100000</v>
+      </c>
+      <c r="F9" s="18" t="s">
+        <v>49</v>
+      </c>
       <c r="G9" s="20"/>
       <c r="H9" s="20"/>
       <c r="I9" s="19"/>
       <c r="J9" s="18"/>
-      <c r="K9" s="18"/>
-      <c r="L9" s="18"/>
-      <c r="M9" s="18"/>
+      <c r="K9" s="18" t="s">
+        <v>125</v>
+      </c>
+      <c r="L9" s="18" t="s">
+        <v>51</v>
+      </c>
+      <c r="M9" s="18" t="s">
+        <v>126</v>
+      </c>
       <c r="N9" s="18"/>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
@@ -1575,7 +1732,7 @@
       <c r="D28" s="2"/>
       <c r="E28" s="15">
         <f>SUMIFS(E6:E25,F6:F25,"&lt;&gt;Refusé")</f>
-        <v>0</v>
+        <v>132000</v>
       </c>
     </row>
     <row r="29" spans="1:14" ht="13" x14ac:dyDescent="0.3">
@@ -1639,11 +1796,11 @@
         <v>62</v>
       </c>
       <c r="C35" s="13">
-        <f>SUMIFS($E$6:$E$25,$B$6:$B$25,B35,$F$6:$F$25,"&lt;&gt;Refusé")</f>
-        <v>0</v>
+        <f t="shared" ref="C35:C41" si="0">SUMIFS($E$6:$E$25,$B$6:$B$25,B35,$F$6:$F$25,"&lt;&gt;Refusé")</f>
+        <v>7000</v>
       </c>
       <c r="D35" s="13">
-        <f>SUMIFS($H$6:$H$25,$B$6:$B$25,B35,$F$6:$F$25,"Fonds reçus")</f>
+        <f t="shared" ref="D35:D41" si="1">SUMIFS($H$6:$H$25,$B$6:$B$25,B35,$F$6:$F$25,"Fonds reçus")</f>
         <v>0</v>
       </c>
     </row>
@@ -1652,11 +1809,11 @@
         <v>63</v>
       </c>
       <c r="C36" s="13">
-        <f>SUMIFS($E$6:$E$25,$B$6:$B$25,B36,$F$6:$F$25,"&lt;&gt;Refusé")</f>
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>100000</v>
       </c>
       <c r="D36" s="13">
-        <f>SUMIFS($H$6:$H$25,$B$6:$B$25,B36,$F$6:$F$25,"Fonds reçus")</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -1665,11 +1822,11 @@
         <v>64</v>
       </c>
       <c r="C37" s="13">
-        <f>SUMIFS($E$6:$E$25,$B$6:$B$25,B37,$F$6:$F$25,"&lt;&gt;Refusé")</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="D37" s="13">
-        <f>SUMIFS($H$6:$H$25,$B$6:$B$25,B37,$F$6:$F$25,"Fonds reçus")</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -1678,11 +1835,11 @@
         <v>45</v>
       </c>
       <c r="C38" s="13">
-        <f>SUMIFS($E$6:$E$25,$B$6:$B$25,B38,$F$6:$F$25,"&lt;&gt;Refusé")</f>
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>20000</v>
       </c>
       <c r="D38" s="13">
-        <f>SUMIFS($H$6:$H$25,$B$6:$B$25,B38,$F$6:$F$25,"Fonds reçus")</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -1691,11 +1848,11 @@
         <v>65</v>
       </c>
       <c r="C39" s="13">
-        <f>SUMIFS($E$6:$E$25,$B$6:$B$25,B39,$F$6:$F$25,"&lt;&gt;Refusé")</f>
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>5000</v>
       </c>
       <c r="D39" s="13">
-        <f>SUMIFS($H$6:$H$25,$B$6:$B$25,B39,$F$6:$F$25,"Fonds reçus")</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -1704,11 +1861,11 @@
         <v>66</v>
       </c>
       <c r="C40" s="13">
-        <f>SUMIFS($E$6:$E$25,$B$6:$B$25,B40,$F$6:$F$25,"&lt;&gt;Refusé")</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="D40" s="13">
-        <f>SUMIFS($H$6:$H$25,$B$6:$B$25,B40,$F$6:$F$25,"Fonds reçus")</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -1717,11 +1874,11 @@
         <v>67</v>
       </c>
       <c r="C41" s="13">
-        <f>SUMIFS($E$6:$E$25,$B$6:$B$25,B41,$F$6:$F$25,"&lt;&gt;Refusé")</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="D41" s="13">
-        <f>SUMIFS($H$6:$H$25,$B$6:$B$25,B41,$F$6:$F$25,"Fonds reçus")</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -1813,23 +1970,39 @@
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A5" s="8"/>
-      <c r="B5" s="8"/>
-      <c r="C5" s="10"/>
-      <c r="D5" s="21"/>
-      <c r="E5" s="22"/>
+      <c r="A5" s="8">
+        <v>2</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>118</v>
+      </c>
+      <c r="C5" s="10">
+        <v>20000</v>
+      </c>
+      <c r="D5" s="21">
+        <v>0</v>
+      </c>
+      <c r="E5" s="22">
+        <v>60</v>
+      </c>
       <c r="F5" s="23">
         <f t="shared" ref="F5:F14" si="0">IF(AND(C5&gt;0,E5&gt;0),IF(D5=0,C5/E5,PMT(D5/12,E5,-C5)),0)</f>
-        <v>0</v>
+        <v>333.33333333333331</v>
       </c>
       <c r="G5" s="23">
         <f t="shared" ref="G5:G14" si="1">IF(F5&gt;0,F5*E5-C5,0)</f>
         <v>0</v>
       </c>
       <c r="H5" s="9"/>
-      <c r="I5" s="8"/>
-      <c r="J5" s="8"/>
-      <c r="K5" s="8"/>
+      <c r="I5" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="J5" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="K5" s="8" t="s">
+        <v>128</v>
+      </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="8"/>
@@ -2009,13 +2182,13 @@
       </c>
       <c r="C15" s="15">
         <f>SUM(C5:C14)</f>
-        <v>0</v>
+        <v>20000</v>
       </c>
       <c r="D15" s="2"/>
       <c r="E15" s="2"/>
       <c r="F15" s="24">
         <f>SUM(F5:F14)</f>
-        <v>0</v>
+        <v>333.33333333333331</v>
       </c>
       <c r="G15" s="24">
         <f>SUM(G5:G14)</f>
@@ -2073,15 +2246,19 @@
       <c r="A3" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="B3" s="9"/>
+      <c r="B3" s="9">
+        <v>46327</v>
+      </c>
       <c r="C3" s="25" t="s">
         <v>84</v>
       </c>
-      <c r="D3" s="26"/>
-      <c r="E3" s="27"/>
-      <c r="F3" s="27"/>
-      <c r="G3" s="27"/>
-      <c r="H3" s="28"/>
+      <c r="D3" s="33" t="s">
+        <v>129</v>
+      </c>
+      <c r="E3" s="34"/>
+      <c r="F3" s="34"/>
+      <c r="G3" s="34"/>
+      <c r="H3" s="35"/>
     </row>
     <row r="5" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
@@ -2116,140 +2293,252 @@
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A6" s="8"/>
-      <c r="B6" s="8"/>
-      <c r="C6" s="22"/>
-      <c r="D6" s="29">
+      <c r="A6" s="8" t="s">
+        <v>130</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>131</v>
+      </c>
+      <c r="C6" s="22">
+        <v>1000</v>
+      </c>
+      <c r="D6" s="26">
         <f t="shared" ref="D6:D17" si="0">IF(OR(B6="BSA ou BSPCE non exercés",$C$18-$C$19=0),0,C6/($C$18-$C$19))</f>
-        <v>0</v>
-      </c>
-      <c r="E6" s="29">
+        <v>0.14285714285714285</v>
+      </c>
+      <c r="E6" s="26">
         <f t="shared" ref="E6:E17" si="1">IF($C$18=0,0,C6/$C$18)</f>
-        <v>0</v>
-      </c>
-      <c r="F6" s="10"/>
-      <c r="G6" s="9"/>
-      <c r="H6" s="8"/>
-      <c r="I6" s="8"/>
-      <c r="J6" s="8"/>
+        <v>0.14285714285714285</v>
+      </c>
+      <c r="F6" s="10">
+        <v>1000</v>
+      </c>
+      <c r="G6" s="9">
+        <v>46327</v>
+      </c>
+      <c r="H6" s="8" t="s">
+        <v>132</v>
+      </c>
+      <c r="I6" s="8" t="s">
+        <v>133</v>
+      </c>
+      <c r="J6" s="8" t="s">
+        <v>51</v>
+      </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A7" s="8"/>
-      <c r="B7" s="8"/>
-      <c r="C7" s="22"/>
-      <c r="D7" s="29">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="E7" s="29">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F7" s="10"/>
-      <c r="G7" s="9"/>
-      <c r="H7" s="8"/>
-      <c r="I7" s="8"/>
-      <c r="J7" s="8"/>
+      <c r="A7" s="8" t="s">
+        <v>134</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>131</v>
+      </c>
+      <c r="C7" s="22">
+        <v>1000</v>
+      </c>
+      <c r="D7" s="26">
+        <f t="shared" si="0"/>
+        <v>0.14285714285714285</v>
+      </c>
+      <c r="E7" s="26">
+        <f t="shared" si="1"/>
+        <v>0.14285714285714285</v>
+      </c>
+      <c r="F7" s="10">
+        <v>1000</v>
+      </c>
+      <c r="G7" s="9">
+        <v>46327</v>
+      </c>
+      <c r="H7" s="8" t="s">
+        <v>132</v>
+      </c>
+      <c r="I7" s="8" t="s">
+        <v>133</v>
+      </c>
+      <c r="J7" s="8" t="s">
+        <v>51</v>
+      </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A8" s="8"/>
-      <c r="B8" s="8"/>
-      <c r="C8" s="22"/>
-      <c r="D8" s="29">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="E8" s="29">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F8" s="10"/>
-      <c r="G8" s="9"/>
-      <c r="H8" s="8"/>
-      <c r="I8" s="8"/>
-      <c r="J8" s="8"/>
+      <c r="A8" s="8" t="s">
+        <v>135</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>131</v>
+      </c>
+      <c r="C8" s="22">
+        <v>1000</v>
+      </c>
+      <c r="D8" s="26">
+        <f t="shared" si="0"/>
+        <v>0.14285714285714285</v>
+      </c>
+      <c r="E8" s="26">
+        <f t="shared" si="1"/>
+        <v>0.14285714285714285</v>
+      </c>
+      <c r="F8" s="10">
+        <v>1000</v>
+      </c>
+      <c r="G8" s="9">
+        <v>46327</v>
+      </c>
+      <c r="H8" s="8" t="s">
+        <v>132</v>
+      </c>
+      <c r="I8" s="8" t="s">
+        <v>133</v>
+      </c>
+      <c r="J8" s="8" t="s">
+        <v>51</v>
+      </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A9" s="8"/>
-      <c r="B9" s="8"/>
-      <c r="C9" s="22"/>
-      <c r="D9" s="29">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="E9" s="29">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F9" s="10"/>
-      <c r="G9" s="9"/>
-      <c r="H9" s="8"/>
-      <c r="I9" s="8"/>
-      <c r="J9" s="8"/>
+      <c r="A9" s="8" t="s">
+        <v>136</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>131</v>
+      </c>
+      <c r="C9" s="22">
+        <v>1000</v>
+      </c>
+      <c r="D9" s="26">
+        <f t="shared" si="0"/>
+        <v>0.14285714285714285</v>
+      </c>
+      <c r="E9" s="26">
+        <f t="shared" si="1"/>
+        <v>0.14285714285714285</v>
+      </c>
+      <c r="F9" s="10">
+        <v>1000</v>
+      </c>
+      <c r="G9" s="9">
+        <v>46327</v>
+      </c>
+      <c r="H9" s="8" t="s">
+        <v>132</v>
+      </c>
+      <c r="I9" s="8" t="s">
+        <v>133</v>
+      </c>
+      <c r="J9" s="8" t="s">
+        <v>51</v>
+      </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A10" s="8"/>
-      <c r="B10" s="8"/>
-      <c r="C10" s="22"/>
-      <c r="D10" s="29">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="E10" s="29">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F10" s="10"/>
-      <c r="G10" s="9"/>
-      <c r="H10" s="8"/>
-      <c r="I10" s="8"/>
-      <c r="J10" s="8"/>
+      <c r="A10" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>131</v>
+      </c>
+      <c r="C10" s="22">
+        <v>1000</v>
+      </c>
+      <c r="D10" s="26">
+        <f t="shared" si="0"/>
+        <v>0.14285714285714285</v>
+      </c>
+      <c r="E10" s="26">
+        <f t="shared" si="1"/>
+        <v>0.14285714285714285</v>
+      </c>
+      <c r="F10" s="10">
+        <v>1000</v>
+      </c>
+      <c r="G10" s="9">
+        <v>46327</v>
+      </c>
+      <c r="H10" s="8" t="s">
+        <v>132</v>
+      </c>
+      <c r="I10" s="8" t="s">
+        <v>133</v>
+      </c>
+      <c r="J10" s="8" t="s">
+        <v>51</v>
+      </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A11" s="8"/>
-      <c r="B11" s="8"/>
-      <c r="C11" s="22"/>
-      <c r="D11" s="29">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="E11" s="29">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F11" s="10"/>
-      <c r="G11" s="9"/>
-      <c r="H11" s="8"/>
-      <c r="I11" s="8"/>
-      <c r="J11" s="8"/>
+      <c r="A11" s="8" t="s">
+        <v>138</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>131</v>
+      </c>
+      <c r="C11" s="22">
+        <v>1000</v>
+      </c>
+      <c r="D11" s="26">
+        <f t="shared" si="0"/>
+        <v>0.14285714285714285</v>
+      </c>
+      <c r="E11" s="26">
+        <f t="shared" si="1"/>
+        <v>0.14285714285714285</v>
+      </c>
+      <c r="F11" s="10">
+        <v>1000</v>
+      </c>
+      <c r="G11" s="9">
+        <v>46327</v>
+      </c>
+      <c r="H11" s="8" t="s">
+        <v>132</v>
+      </c>
+      <c r="I11" s="8" t="s">
+        <v>133</v>
+      </c>
+      <c r="J11" s="8" t="s">
+        <v>51</v>
+      </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A12" s="8"/>
-      <c r="B12" s="8"/>
-      <c r="C12" s="22"/>
-      <c r="D12" s="29">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="E12" s="29">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F12" s="10"/>
-      <c r="G12" s="9"/>
-      <c r="H12" s="8"/>
-      <c r="I12" s="8"/>
-      <c r="J12" s="8"/>
+      <c r="A12" s="8" t="s">
+        <v>139</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>131</v>
+      </c>
+      <c r="C12" s="22">
+        <v>1000</v>
+      </c>
+      <c r="D12" s="26">
+        <f t="shared" si="0"/>
+        <v>0.14285714285714285</v>
+      </c>
+      <c r="E12" s="26">
+        <f t="shared" si="1"/>
+        <v>0.14285714285714285</v>
+      </c>
+      <c r="F12" s="10">
+        <v>1000</v>
+      </c>
+      <c r="G12" s="9">
+        <v>46327</v>
+      </c>
+      <c r="H12" s="8" t="s">
+        <v>132</v>
+      </c>
+      <c r="I12" s="8" t="s">
+        <v>133</v>
+      </c>
+      <c r="J12" s="8" t="s">
+        <v>51</v>
+      </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="8"/>
       <c r="B13" s="8"/>
       <c r="C13" s="22"/>
-      <c r="D13" s="29">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="E13" s="29">
+      <c r="D13" s="26">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="E13" s="26">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -2263,11 +2552,11 @@
       <c r="A14" s="8"/>
       <c r="B14" s="8"/>
       <c r="C14" s="22"/>
-      <c r="D14" s="29">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="E14" s="29">
+      <c r="D14" s="26">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="E14" s="26">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -2281,11 +2570,11 @@
       <c r="A15" s="8"/>
       <c r="B15" s="8"/>
       <c r="C15" s="22"/>
-      <c r="D15" s="29">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="E15" s="29">
+      <c r="D15" s="26">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="E15" s="26">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -2299,11 +2588,11 @@
       <c r="A16" s="8"/>
       <c r="B16" s="8"/>
       <c r="C16" s="22"/>
-      <c r="D16" s="29">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="E16" s="29">
+      <c r="D16" s="26">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="E16" s="26">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -2317,11 +2606,11 @@
       <c r="A17" s="8"/>
       <c r="B17" s="8"/>
       <c r="C17" s="22"/>
-      <c r="D17" s="29">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="E17" s="29">
+      <c r="D17" s="26">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="E17" s="26">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -2338,19 +2627,19 @@
       <c r="B18" s="2"/>
       <c r="C18" s="16">
         <f>SUM(C6:C17)</f>
-        <v>0</v>
-      </c>
-      <c r="D18" s="30">
+        <v>7000</v>
+      </c>
+      <c r="D18" s="27">
         <f>SUM(D6:D17)</f>
-        <v>0</v>
-      </c>
-      <c r="E18" s="30">
+        <v>0.99999999999999978</v>
+      </c>
+      <c r="E18" s="27">
         <f>SUM(E6:E17)</f>
-        <v>0</v>
+        <v>0.99999999999999978</v>
       </c>
       <c r="F18" s="15">
         <f>SUM(F6:F17)</f>
-        <v>0</v>
+        <v>7000</v>
       </c>
     </row>
     <row r="19" spans="1:10" ht="13" x14ac:dyDescent="0.3">
@@ -2398,7 +2687,7 @@
       </c>
     </row>
     <row r="2" spans="1:5" ht="13" x14ac:dyDescent="0.3">
-      <c r="A2" s="31" t="s">
+      <c r="A2" s="28" t="s">
         <v>96</v>
       </c>
     </row>
@@ -2420,33 +2709,51 @@
       <c r="A5" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="B5" s="10"/>
-      <c r="C5" s="8"/>
-      <c r="D5" s="8"/>
+      <c r="B5" s="10">
+        <v>400000</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>141</v>
+      </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="B6" s="10"/>
-      <c r="C6" s="8"/>
-      <c r="D6" s="8"/>
+      <c r="B6" s="10">
+        <v>100000</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>142</v>
+      </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="B7" s="32"/>
-      <c r="C7" s="8"/>
-      <c r="D7" s="8"/>
+      <c r="B7" s="29" t="s">
+        <v>140</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>143</v>
+      </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="B8" s="34">
+      <c r="B8" s="31">
         <f>'Table de capitalisation'!C18</f>
-        <v>0</v>
+        <v>7000</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
@@ -2455,7 +2762,7 @@
       </c>
       <c r="B9" s="23">
         <f>IF(B8&gt;0,B5/B8,0)</f>
-        <v>0</v>
+        <v>57.142857142857146</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
@@ -2464,7 +2771,7 @@
       </c>
       <c r="B10" s="14">
         <f>IF(B9&gt;0,ROUND(B6/B9,0),0)</f>
-        <v>0</v>
+        <v>1750</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
@@ -2473,16 +2780,16 @@
       </c>
       <c r="B11" s="13">
         <f>B5+B6</f>
-        <v>0</v>
+        <v>500000</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="B12" s="29">
+      <c r="B12" s="26">
         <f>IF(B11&gt;0,B6/B11,0)</f>
-        <v>0</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -2503,169 +2810,169 @@
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" s="33" t="str">
+      <c r="A15" s="30" t="str">
         <f>IF('Table de capitalisation'!A6="","",'Table de capitalisation'!A6)</f>
-        <v/>
-      </c>
-      <c r="B15" s="34">
+        <v>Associé fondateur (Direction)</v>
+      </c>
+      <c r="B15" s="31">
         <f>'Table de capitalisation'!C6</f>
-        <v>0</v>
-      </c>
-      <c r="C15" s="29">
+        <v>1000</v>
+      </c>
+      <c r="C15" s="26">
         <f t="shared" ref="C15:C26" si="0">IF($B$8=0,0,B15/$B$8)</f>
-        <v>0</v>
+        <v>0.14285714285714285</v>
       </c>
       <c r="D15" s="14">
         <f t="shared" ref="D15:D26" si="1">B15</f>
-        <v>0</v>
-      </c>
-      <c r="E15" s="29">
+        <v>1000</v>
+      </c>
+      <c r="E15" s="26">
         <f t="shared" ref="E15:E26" si="2">IF($D$28=0,0,D15/$D$28)</f>
-        <v>0</v>
+        <v>0.11428571428571428</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" s="33" t="str">
+      <c r="A16" s="30" t="str">
         <f>IF('Table de capitalisation'!A7="","",'Table de capitalisation'!A7)</f>
-        <v/>
-      </c>
-      <c r="B16" s="34">
+        <v>Associé fondateur (Finance)</v>
+      </c>
+      <c r="B16" s="31">
         <f>'Table de capitalisation'!C7</f>
-        <v>0</v>
-      </c>
-      <c r="C16" s="29">
-        <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1000</v>
+      </c>
+      <c r="C16" s="26">
+        <f t="shared" si="0"/>
+        <v>0.14285714285714285</v>
       </c>
       <c r="D16" s="14">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="E16" s="29">
+        <v>1000</v>
+      </c>
+      <c r="E16" s="26">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>0.11428571428571428</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" s="33" t="str">
+      <c r="A17" s="30" t="str">
         <f>IF('Table de capitalisation'!A8="","",'Table de capitalisation'!A8)</f>
-        <v/>
-      </c>
-      <c r="B17" s="34">
+        <v>Associé fondateur (Marketing)</v>
+      </c>
+      <c r="B17" s="31">
         <f>'Table de capitalisation'!C8</f>
-        <v>0</v>
-      </c>
-      <c r="C17" s="29">
-        <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1000</v>
+      </c>
+      <c r="C17" s="26">
+        <f t="shared" si="0"/>
+        <v>0.14285714285714285</v>
       </c>
       <c r="D17" s="14">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="E17" s="29">
+        <v>1000</v>
+      </c>
+      <c r="E17" s="26">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>0.11428571428571428</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" s="33" t="str">
+      <c r="A18" s="30" t="str">
         <f>IF('Table de capitalisation'!A9="","",'Table de capitalisation'!A9)</f>
-        <v/>
-      </c>
-      <c r="B18" s="34">
+        <v>Associé fondateur (Ventes)</v>
+      </c>
+      <c r="B18" s="31">
         <f>'Table de capitalisation'!C9</f>
-        <v>0</v>
-      </c>
-      <c r="C18" s="29">
-        <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1000</v>
+      </c>
+      <c r="C18" s="26">
+        <f t="shared" si="0"/>
+        <v>0.14285714285714285</v>
       </c>
       <c r="D18" s="14">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="E18" s="29">
+        <v>1000</v>
+      </c>
+      <c r="E18" s="26">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>0.11428571428571428</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A19" s="33" t="str">
+      <c r="A19" s="30" t="str">
         <f>IF('Table de capitalisation'!A10="","",'Table de capitalisation'!A10)</f>
-        <v/>
-      </c>
-      <c r="B19" s="34">
+        <v>Associé fondateur (Produit)</v>
+      </c>
+      <c r="B19" s="31">
         <f>'Table de capitalisation'!C10</f>
-        <v>0</v>
-      </c>
-      <c r="C19" s="29">
-        <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1000</v>
+      </c>
+      <c r="C19" s="26">
+        <f t="shared" si="0"/>
+        <v>0.14285714285714285</v>
       </c>
       <c r="D19" s="14">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="E19" s="29">
+        <v>1000</v>
+      </c>
+      <c r="E19" s="26">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>0.11428571428571428</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" s="33" t="str">
+      <c r="A20" s="30" t="str">
         <f>IF('Table de capitalisation'!A11="","",'Table de capitalisation'!A11)</f>
-        <v/>
-      </c>
-      <c r="B20" s="34">
+        <v>Associé fondateur (Opérations)</v>
+      </c>
+      <c r="B20" s="31">
         <f>'Table de capitalisation'!C11</f>
-        <v>0</v>
-      </c>
-      <c r="C20" s="29">
-        <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1000</v>
+      </c>
+      <c r="C20" s="26">
+        <f t="shared" si="0"/>
+        <v>0.14285714285714285</v>
       </c>
       <c r="D20" s="14">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="E20" s="29">
+        <v>1000</v>
+      </c>
+      <c r="E20" s="26">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>0.11428571428571428</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A21" s="33" t="str">
+      <c r="A21" s="30" t="str">
         <f>IF('Table de capitalisation'!A12="","",'Table de capitalisation'!A12)</f>
-        <v/>
-      </c>
-      <c r="B21" s="34">
+        <v>Associé fondateur (Juridique)</v>
+      </c>
+      <c r="B21" s="31">
         <f>'Table de capitalisation'!C12</f>
-        <v>0</v>
-      </c>
-      <c r="C21" s="29">
-        <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1000</v>
+      </c>
+      <c r="C21" s="26">
+        <f t="shared" si="0"/>
+        <v>0.14285714285714285</v>
       </c>
       <c r="D21" s="14">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="E21" s="29">
+        <v>1000</v>
+      </c>
+      <c r="E21" s="26">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>0.11428571428571428</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A22" s="33" t="str">
+      <c r="A22" s="30" t="str">
         <f>IF('Table de capitalisation'!A13="","",'Table de capitalisation'!A13)</f>
         <v/>
       </c>
-      <c r="B22" s="34">
+      <c r="B22" s="31">
         <f>'Table de capitalisation'!C13</f>
         <v>0</v>
       </c>
-      <c r="C22" s="29">
+      <c r="C22" s="26">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -2673,21 +2980,21 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="E22" s="29">
+      <c r="E22" s="26">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A23" s="33" t="str">
+      <c r="A23" s="30" t="str">
         <f>IF('Table de capitalisation'!A14="","",'Table de capitalisation'!A14)</f>
         <v/>
       </c>
-      <c r="B23" s="34">
+      <c r="B23" s="31">
         <f>'Table de capitalisation'!C14</f>
         <v>0</v>
       </c>
-      <c r="C23" s="29">
+      <c r="C23" s="26">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -2695,21 +3002,21 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="E23" s="29">
+      <c r="E23" s="26">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A24" s="33" t="str">
+      <c r="A24" s="30" t="str">
         <f>IF('Table de capitalisation'!A15="","",'Table de capitalisation'!A15)</f>
         <v/>
       </c>
-      <c r="B24" s="34">
+      <c r="B24" s="31">
         <f>'Table de capitalisation'!C15</f>
         <v>0</v>
       </c>
-      <c r="C24" s="29">
+      <c r="C24" s="26">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -2717,21 +3024,21 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="E24" s="29">
+      <c r="E24" s="26">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A25" s="33" t="str">
+      <c r="A25" s="30" t="str">
         <f>IF('Table de capitalisation'!A16="","",'Table de capitalisation'!A16)</f>
         <v/>
       </c>
-      <c r="B25" s="34">
+      <c r="B25" s="31">
         <f>'Table de capitalisation'!C16</f>
         <v>0</v>
       </c>
-      <c r="C25" s="29">
+      <c r="C25" s="26">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -2739,21 +3046,21 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="E25" s="29">
+      <c r="E25" s="26">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A26" s="33" t="str">
+      <c r="A26" s="30" t="str">
         <f>IF('Table de capitalisation'!A17="","",'Table de capitalisation'!A17)</f>
         <v/>
       </c>
-      <c r="B26" s="34">
+      <c r="B26" s="31">
         <f>'Table de capitalisation'!C17</f>
         <v>0</v>
       </c>
-      <c r="C26" s="29">
+      <c r="C26" s="26">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -2761,7 +3068,7 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="E26" s="29">
+      <c r="E26" s="26">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
@@ -2769,42 +3076,42 @@
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="12" t="str">
         <f>IF(B7="","Nouveaux investisseurs",B7)</f>
-        <v>Nouveaux investisseurs</v>
+        <v>Business angels, dont un associé gastronomique (H)</v>
       </c>
       <c r="B27" s="14">
         <v>0</v>
       </c>
-      <c r="C27" s="29">
+      <c r="C27" s="26">
         <v>0</v>
       </c>
       <c r="D27" s="14">
         <f>B10</f>
-        <v>0</v>
-      </c>
-      <c r="E27" s="29">
+        <v>1750</v>
+      </c>
+      <c r="E27" s="26">
         <f>IF($D$28=0,0,D27/$D$28)</f>
-        <v>0</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="13" x14ac:dyDescent="0.3">
-      <c r="A28" s="35" t="s">
+      <c r="A28" s="32" t="s">
         <v>79</v>
       </c>
       <c r="B28" s="16">
         <f>SUM(B15:B27)</f>
-        <v>0</v>
-      </c>
-      <c r="C28" s="30">
+        <v>7000</v>
+      </c>
+      <c r="C28" s="27">
         <f>SUM(C15:C27)</f>
-        <v>0</v>
+        <v>0.99999999999999978</v>
       </c>
       <c r="D28" s="16">
         <f>SUM(D15:D27)</f>
-        <v>0</v>
-      </c>
-      <c r="E28" s="30">
+        <v>8750</v>
+      </c>
+      <c r="E28" s="27">
         <f>SUM(E15:E27)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="13" x14ac:dyDescent="0.3">

</xml_diff>